<commit_message>
added sprint plan to project_plan.xlsx ; created mvp workflow doc ; created questionnaire output json example
</commit_message>
<xml_diff>
--- a/project_plan.xlsx
+++ b/project_plan.xlsx
@@ -3,19 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CA52FD-68F5-461A-91AA-494660226D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA007FAD-25E6-4D83-859A-BCF323A566AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
+    <sheet name="Sprint Plan" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="88">
   <si>
     <t>Gain access to the Dev pannel of Shopify website for CelRevive from client.</t>
   </si>
@@ -201,12 +202,263 @@
       <t xml:space="preserve"> — no new table needed</t>
     </r>
   </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Add exclusion table</t>
+  </si>
+  <si>
+    <t>Design schema (allergen/exclusion master + active link table)</t>
+  </si>
+  <si>
+    <t>Map questionnaire allergen field → exclusion table (structured, not free-text)</t>
+  </si>
+  <si>
+    <t>Write DDL migration</t>
+  </si>
+  <si>
+    <t>Seed exclusion data from workbook/domain input</t>
+  </si>
+  <si>
+    <t>Write QA query to validate coverage (e.g. every active has been assessed against every known allergen category)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image Preprocessing &amp; Quality Validation </t>
+  </si>
+  <si>
+    <t>Define acceptance thresholds (blur, lighting,resolution)</t>
+  </si>
+  <si>
+    <t>Implement preprocessing pipeline</t>
+  </si>
+  <si>
+    <t>Quality gate + reject/retry module</t>
+  </si>
+  <si>
+    <t>Vision LLM Concern Extraction</t>
+  </si>
+  <si>
+    <t>Define prompt structure</t>
+  </si>
+  <si>
+    <t>Questionnaire Concern Extraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concern Fusion </t>
+  </si>
+  <si>
+    <t>Fuse questionnaire &amp; image skin detected skin concerns using OR  logic i.e
+skin_concerns = questionnaire_concerns OR image_concerns</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Update </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>session_skin_concern_score</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> table</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">join </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>concern_benefit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>active_benefit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>score+base_active_compatability</t>
+    </r>
+  </si>
+  <si>
+    <t>Apply exclusion filter</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Define JSON package shape for LLM call - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>shortlist_json</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Formulation LLM Call </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Draft prompt template consuming </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">shortlist_json </t>
+    </r>
+  </si>
+  <si>
+    <t>Define output Json Schema</t>
+  </si>
+  <si>
+    <t>Work Serial</t>
+  </si>
+  <si>
+    <t>Desginated Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend Sprint </t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>LLM Interaction auditing</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Define </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>audit_log</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> payload shape per event_type (image, questionnaire,formulation)</t>
+    </r>
+  </si>
+  <si>
+    <t>Implement logging calls at each LLM touchpoint</t>
+  </si>
+  <si>
+    <t>Define final response schema (formulation,actives,bases,explanation, formulation_id,etc)</t>
+  </si>
+  <si>
+    <t>Implement DB -&gt; Json serialization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Define error/fallback response </t>
+  </si>
+  <si>
+    <t>Shopify integration test</t>
+  </si>
+  <si>
+    <t>Work Sub Serial</t>
+  </si>
+  <si>
+    <t>Sprint Serial</t>
+  </si>
+  <si>
+    <t>SQL Candidate Shortlist Query (Optional)</t>
+  </si>
+  <si>
+    <t>Audit final candidate table</t>
+  </si>
+  <si>
+    <t>Sprint Start</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Define output JSON structure </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -216,13 +468,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -248,7 +493,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -273,8 +518,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -297,11 +554,91 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -312,22 +649,10 @@
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -336,16 +661,61 @@
     <xf numFmtId="16" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -833,20 +1203,20 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="12" customFormat="1" ht="28.8">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10">
+    <row r="10" spans="1:7" s="10" customFormat="1" ht="28.8">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6">
         <v>9</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="10"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="10" t="s">
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="11"/>
+      <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" ht="43.2">
       <c r="B11" s="1">
@@ -888,18 +1258,18 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="13" spans="1:7" s="12" customFormat="1">
-      <c r="A13" s="10"/>
-      <c r="B13" s="10">
+    <row r="13" spans="1:7" s="10" customFormat="1">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6">
         <v>11</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="10"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="11"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1" ht="57.6">
       <c r="B14" s="4">
@@ -921,7 +1291,7 @@
         <v>46248</v>
       </c>
     </row>
-    <row r="15" spans="1:7" s="13" customFormat="1" ht="28.8">
+    <row r="15" spans="1:7" s="11" customFormat="1" ht="28.8">
       <c r="A15" s="8"/>
       <c r="B15" s="8">
         <v>12</v>
@@ -971,7 +1341,7 @@
         <v>46255</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="14" customFormat="1" ht="72">
+    <row r="18" spans="1:7" s="10" customFormat="1" ht="72">
       <c r="A18" s="6"/>
       <c r="B18" s="6">
         <v>14</v>
@@ -986,7 +1356,7 @@
       </c>
       <c r="G18" s="7"/>
     </row>
-    <row r="19" spans="1:7" s="14" customFormat="1" ht="28.8">
+    <row r="19" spans="1:7" s="10" customFormat="1" ht="28.8">
       <c r="A19" s="6"/>
       <c r="B19" s="6">
         <v>15</v>
@@ -1086,7 +1456,7 @@
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="12" t="s">
         <v>46</v>
       </c>
       <c r="G24" s="7"/>
@@ -1104,7 +1474,7 @@
       <c r="E25" s="3">
         <v>46258</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="10" t="s">
         <v>25</v>
       </c>
       <c r="G25" s="3">
@@ -1115,4 +1485,463 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B28C61C-1A55-4D93-BE97-335A9CE60726}">
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" style="14" customWidth="1"/>
+    <col min="3" max="3" width="15.109375" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="33.33203125" style="13" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" customWidth="1"/>
+    <col min="8" max="8" width="16.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="32"/>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="I2" s="23" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="58.8" customHeight="1">
+      <c r="A3" s="24"/>
+      <c r="B3" s="28">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="I3" s="25"/>
+    </row>
+    <row r="4" spans="1:9" ht="54.6" customHeight="1">
+      <c r="A4" s="24"/>
+      <c r="B4" s="28"/>
+      <c r="C4">
+        <v>1.2</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="25"/>
+    </row>
+    <row r="5" spans="1:9" ht="33.6" customHeight="1">
+      <c r="A5" s="24"/>
+      <c r="B5" s="28"/>
+      <c r="C5">
+        <v>1.3</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="I5" s="25"/>
+    </row>
+    <row r="6" spans="1:9" ht="26.4" customHeight="1">
+      <c r="A6" s="24"/>
+      <c r="B6" s="28"/>
+      <c r="C6">
+        <v>1.4</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="25"/>
+    </row>
+    <row r="7" spans="1:9" ht="72.599999999999994" customHeight="1">
+      <c r="A7" s="24"/>
+      <c r="B7" s="28"/>
+      <c r="C7">
+        <v>1.5</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" s="25"/>
+    </row>
+    <row r="8" spans="1:9" ht="28.8">
+      <c r="A8" s="24"/>
+      <c r="B8" s="28">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>2.1</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="25"/>
+    </row>
+    <row r="9" spans="1:9" ht="28.8">
+      <c r="A9" s="24"/>
+      <c r="B9" s="28"/>
+      <c r="C9">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="I9" s="25"/>
+    </row>
+    <row r="10" spans="1:9" ht="28.8">
+      <c r="A10" s="24"/>
+      <c r="B10" s="28"/>
+      <c r="C10">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="I10" s="25"/>
+    </row>
+    <row r="11" spans="1:9" ht="28.8">
+      <c r="A11" s="24"/>
+      <c r="B11" s="28">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3.1</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="I11" s="25"/>
+    </row>
+    <row r="12" spans="1:9" ht="28.8">
+      <c r="A12" s="24"/>
+      <c r="B12" s="28"/>
+      <c r="C12">
+        <v>3.2</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="I12" s="25"/>
+    </row>
+    <row r="13" spans="1:9" ht="28.8">
+      <c r="A13" s="24"/>
+      <c r="B13" s="28">
+        <v>4</v>
+      </c>
+      <c r="C13">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="I13" s="25"/>
+    </row>
+    <row r="14" spans="1:9" ht="28.8">
+      <c r="A14" s="24"/>
+      <c r="B14" s="28"/>
+      <c r="C14">
+        <v>4.2</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="I14" s="25"/>
+    </row>
+    <row r="15" spans="1:9" ht="86.4">
+      <c r="A15" s="24"/>
+      <c r="B15" s="28">
+        <v>5</v>
+      </c>
+      <c r="C15">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="I15" s="25"/>
+    </row>
+    <row r="16" spans="1:9" ht="28.8">
+      <c r="A16" s="24"/>
+      <c r="B16" s="28"/>
+      <c r="C16">
+        <v>5.2</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="I16" s="25"/>
+    </row>
+    <row r="17" spans="1:9" ht="28.8">
+      <c r="A17" s="24"/>
+      <c r="B17" s="28">
+        <v>6</v>
+      </c>
+      <c r="C17">
+        <v>6.1</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="I17" s="25"/>
+    </row>
+    <row r="18" spans="1:9" ht="28.8">
+      <c r="A18" s="24"/>
+      <c r="B18" s="28"/>
+      <c r="C18">
+        <v>6.2</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="I18" s="25"/>
+    </row>
+    <row r="19" spans="1:9" ht="43.8" customHeight="1">
+      <c r="A19" s="24"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="18">
+        <v>6.3</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19" s="25"/>
+    </row>
+    <row r="20" spans="1:9" ht="28.8">
+      <c r="A20" s="24"/>
+      <c r="B20" s="28"/>
+      <c r="C20">
+        <v>6.4</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="I20" s="25"/>
+    </row>
+    <row r="21" spans="1:9" ht="28.8">
+      <c r="A21" s="24"/>
+      <c r="B21" s="28">
+        <v>7</v>
+      </c>
+      <c r="C21">
+        <v>7.1</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="I21" s="25"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="24"/>
+      <c r="B22" s="28"/>
+      <c r="C22">
+        <v>7.2</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22" s="25"/>
+    </row>
+    <row r="23" spans="1:9" ht="43.2">
+      <c r="A23" s="24"/>
+      <c r="B23" s="28">
+        <v>8</v>
+      </c>
+      <c r="C23">
+        <v>8.1</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="I23" s="25"/>
+    </row>
+    <row r="24" spans="1:9" ht="28.8">
+      <c r="A24" s="24"/>
+      <c r="B24" s="28"/>
+      <c r="C24">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="I24" s="25"/>
+    </row>
+    <row r="25" spans="1:9" ht="43.2">
+      <c r="A25" s="24"/>
+      <c r="B25" s="28">
+        <v>9</v>
+      </c>
+      <c r="C25">
+        <v>9.1</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="I25" s="25"/>
+    </row>
+    <row r="26" spans="1:9" ht="28.8">
+      <c r="A26" s="24"/>
+      <c r="B26" s="28"/>
+      <c r="C26">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="I26" s="25"/>
+    </row>
+    <row r="27" spans="1:9" ht="28.8">
+      <c r="A27" s="24"/>
+      <c r="B27" s="28"/>
+      <c r="C27">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="D27" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="I27" s="25"/>
+    </row>
+    <row r="28" spans="1:9" ht="28.8">
+      <c r="A28" s="26"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="20">
+        <v>9.4</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="E28" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="27"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="B25:B28"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B20"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated sprint plan : refer sheet 3
</commit_message>
<xml_diff>
--- a/project_plan.xlsx
+++ b/project_plan.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0CC603-084A-495E-8B76-D4533DDF2B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8E2665-D8D7-4719-A55A-FBF7991E0138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
     <sheet name="Sprint Plan" sheetId="2" r:id="rId2"/>
+    <sheet name="Agile Sprint" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="133">
   <si>
     <t>Gain access to the Dev pannel of Shopify website for CelRevive from client.</t>
   </si>
@@ -560,6 +561,219 @@
       </rPr>
       <t>(vector db query ; no deterministic logic)</t>
     </r>
+  </si>
+  <si>
+    <t>Sprint</t>
+  </si>
+  <si>
+    <t>User Story</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Story Points</t>
+  </si>
+  <si>
+    <t>Designated Team</t>
+  </si>
+  <si>
+    <t>Must</t>
+  </si>
+  <si>
+    <t>Image Preprocessing &amp; Quality</t>
+  </si>
+  <si>
+    <t>Questionnaire concern extraction</t>
+  </si>
+  <si>
+    <t>Should</t>
+  </si>
+  <si>
+    <t>Concern Fusion</t>
+  </si>
+  <si>
+    <t>As a customer, I want the system to shortlist compatible actives and bases based on my combined image and questionnaire concerns, so that only relevant, safe candidates feed into my formulation.</t>
+  </si>
+  <si>
+    <t>As a customer, I want to receive a formulation — recommended
+ actives, bases, dosage and explanation — based on my shortlisted 
+candidates, so that I get a personalised, safe product recommendation.</t>
+  </si>
+  <si>
+    <t>Formulation LLM Call</t>
+  </si>
+  <si>
+    <t>LLM interaction auditing</t>
+  </si>
+  <si>
+    <t>Internal Review</t>
+  </si>
+  <si>
+    <t>Client Review</t>
+  </si>
+  <si>
+    <t>Shopify Integration Feasibility Test</t>
+  </si>
+  <si>
+    <t>Test the feasibility of shopify api integration</t>
+  </si>
+  <si>
+    <t>pending access to client shopify store</t>
+  </si>
+  <si>
+    <t>Quality Testing</t>
+  </si>
+  <si>
+    <t>Create a test dataset</t>
+  </si>
+  <si>
+    <t>Validate System with test dataset</t>
+  </si>
+  <si>
+    <t>MVP_SPRINT_PLAN</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>As a</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> customer,</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> I want to</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> upload a picture of my skin , and after processing receive the detected skin concerns, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>so that</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> the system has a basis for formulation reccomendation(actives)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>As a</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> customer, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>I want to</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> answer a questionnaire, and after processing, receive my detected skin concerns, allergies, contraindications and skin properties (?),</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>so that</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> system understands my entire skin profile for formulation reccomendation ( bases)</t>
+    </r>
+  </si>
+  <si>
+    <t>Response to frontend</t>
+  </si>
+  <si>
+    <t>Return json containing detected skin concerns, allergies , and other relevant properties , to the front end.</t>
+  </si>
+  <si>
+    <t>Expected MVP showcase</t>
+  </si>
+  <si>
+    <t>Expected Skin concern detection showcase</t>
   </si>
 </sst>
 </file>
@@ -608,7 +822,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -645,8 +859,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -669,11 +907,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -756,9 +1040,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -770,10 +1060,88 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1565,20 +1933,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
-      <c r="J1" s="35"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="15" t="s">
@@ -1619,10 +1987,10 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="58.8" customHeight="1">
-      <c r="A3" s="31">
+      <c r="A3" s="33">
         <v>1</v>
       </c>
-      <c r="B3" s="31">
+      <c r="B3" s="33">
         <v>1</v>
       </c>
       <c r="C3">
@@ -1634,25 +2002,25 @@
       <c r="E3" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="33">
+      <c r="F3" s="35">
         <v>46252</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="33" t="s">
         <v>94</v>
       </c>
-      <c r="H3" s="33">
+      <c r="H3" s="35">
         <v>46259</v>
       </c>
-      <c r="I3" s="31" t="s">
+      <c r="I3" s="33" t="s">
         <v>88</v>
       </c>
-      <c r="J3" s="31" t="s">
+      <c r="J3" s="33" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="54.6" customHeight="1">
-      <c r="A4" s="31"/>
-      <c r="B4" s="31"/>
+      <c r="A4" s="33"/>
+      <c r="B4" s="33"/>
       <c r="C4">
         <v>1.2</v>
       </c>
@@ -1662,15 +2030,15 @@
       <c r="E4" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="33"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
     </row>
     <row r="5" spans="1:12" ht="33.6" customHeight="1">
-      <c r="A5" s="31"/>
-      <c r="B5" s="31"/>
+      <c r="A5" s="33"/>
+      <c r="B5" s="33"/>
       <c r="C5">
         <v>1.3</v>
       </c>
@@ -1680,15 +2048,15 @@
       <c r="E5" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="33"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
+      <c r="F5" s="35"/>
+      <c r="G5" s="33"/>
+      <c r="H5" s="33"/>
+      <c r="I5" s="33"/>
+      <c r="J5" s="33"/>
     </row>
     <row r="6" spans="1:12" ht="26.4" customHeight="1">
-      <c r="A6" s="31"/>
-      <c r="B6" s="31"/>
+      <c r="A6" s="33"/>
+      <c r="B6" s="33"/>
       <c r="C6">
         <v>1.4</v>
       </c>
@@ -1698,15 +2066,15 @@
       <c r="E6" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="33"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="33"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="33"/>
     </row>
     <row r="7" spans="1:12" ht="72.599999999999994" customHeight="1">
-      <c r="A7" s="31"/>
-      <c r="B7" s="31"/>
+      <c r="A7" s="33"/>
+      <c r="B7" s="33"/>
       <c r="C7">
         <v>1.5</v>
       </c>
@@ -1716,15 +2084,15 @@
       <c r="E7" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="F7" s="33"/>
-      <c r="G7" s="31"/>
-      <c r="H7" s="31"/>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="31"/>
-      <c r="B8" s="31">
+      <c r="A8" s="33"/>
+      <c r="B8" s="33">
         <v>2</v>
       </c>
       <c r="C8">
@@ -1736,23 +2104,23 @@
       <c r="E8" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="35">
         <v>46252</v>
       </c>
-      <c r="G8" s="31" t="s">
+      <c r="G8" s="33" t="s">
         <v>90</v>
       </c>
-      <c r="H8" s="33">
+      <c r="H8" s="35">
         <v>46258</v>
       </c>
-      <c r="I8" s="31" t="s">
+      <c r="I8" s="33" t="s">
         <v>89</v>
       </c>
-      <c r="J8" s="31"/>
+      <c r="J8" s="33"/>
     </row>
     <row r="9" spans="1:12" ht="28.8">
-      <c r="A9" s="31"/>
-      <c r="B9" s="31"/>
+      <c r="A9" s="33"/>
+      <c r="B9" s="33"/>
       <c r="C9">
         <v>2.2000000000000002</v>
       </c>
@@ -1762,15 +2130,15 @@
       <c r="E9" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="33"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="31"/>
-      <c r="J9" s="31"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
-      <c r="A10" s="31"/>
-      <c r="B10" s="31"/>
+      <c r="A10" s="33"/>
+      <c r="B10" s="33"/>
       <c r="C10">
         <v>2.2999999999999998</v>
       </c>
@@ -1780,15 +2148,15 @@
       <c r="E10" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="33"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="35"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
     </row>
     <row r="11" spans="1:12" ht="28.8">
-      <c r="A11" s="31"/>
-      <c r="B11" s="31">
+      <c r="A11" s="33"/>
+      <c r="B11" s="33">
         <v>3</v>
       </c>
       <c r="C11">
@@ -1800,15 +2168,15 @@
       <c r="E11" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="F11" s="33"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="31"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="33"/>
+      <c r="H11" s="35"/>
+      <c r="I11" s="33"/>
+      <c r="J11" s="33"/>
     </row>
     <row r="12" spans="1:12" ht="28.8">
-      <c r="A12" s="31"/>
-      <c r="B12" s="31"/>
+      <c r="A12" s="33"/>
+      <c r="B12" s="33"/>
       <c r="C12">
         <v>3.2</v>
       </c>
@@ -1830,11 +2198,11 @@
       <c r="I12" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="J12" s="31"/>
+      <c r="J12" s="33"/>
     </row>
     <row r="13" spans="1:12" ht="28.8">
-      <c r="A13" s="31"/>
-      <c r="B13" s="31">
+      <c r="A13" s="33"/>
+      <c r="B13" s="33">
         <v>4</v>
       </c>
       <c r="C13">
@@ -1858,11 +2226,11 @@
       <c r="I13" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="J13" s="31"/>
+      <c r="J13" s="33"/>
     </row>
     <row r="14" spans="1:12" ht="28.8">
-      <c r="A14" s="31"/>
-      <c r="B14" s="31"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="33"/>
       <c r="C14">
         <v>4.2</v>
       </c>
@@ -1884,10 +2252,10 @@
       <c r="I14" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="J14" s="31"/>
+      <c r="J14" s="33"/>
     </row>
     <row r="15" spans="1:12" ht="28.8">
-      <c r="A15" s="31"/>
+      <c r="A15" s="33"/>
       <c r="B15" s="14">
         <v>9</v>
       </c>
@@ -1900,15 +2268,15 @@
       <c r="E15" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="33" t="s">
+      <c r="F15" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
+      <c r="G15" s="35"/>
+      <c r="H15" s="35"/>
       <c r="I15" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="J15" s="31"/>
+      <c r="J15" s="33"/>
       <c r="L15" t="s">
         <v>98</v>
       </c>
@@ -1917,10 +2285,10 @@
       <c r="A16" s="23"/>
       <c r="B16" s="24"/>
       <c r="C16" s="25"/>
-      <c r="D16" s="34" t="s">
+      <c r="D16" s="36" t="s">
         <v>95</v>
       </c>
-      <c r="E16" s="34"/>
+      <c r="E16" s="36"/>
       <c r="F16" s="26">
         <v>46198</v>
       </c>
@@ -1931,10 +2299,10 @@
       <c r="I16" s="24"/>
     </row>
     <row r="17" spans="1:9" ht="86.4">
-      <c r="A17" s="31">
+      <c r="A17" s="33">
         <v>2</v>
       </c>
-      <c r="B17" s="31">
+      <c r="B17" s="33">
         <v>5</v>
       </c>
       <c r="C17">
@@ -1949,19 +2317,19 @@
       <c r="F17" s="21">
         <v>46260</v>
       </c>
-      <c r="G17" s="32" t="s">
+      <c r="G17" s="31" t="s">
         <v>100</v>
       </c>
-      <c r="H17" s="36">
+      <c r="H17" s="32">
         <v>46262</v>
       </c>
-      <c r="I17" s="32" t="s">
+      <c r="I17" s="31" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="28.8">
-      <c r="A18" s="31"/>
-      <c r="B18" s="31"/>
+      <c r="A18" s="33"/>
+      <c r="B18" s="33"/>
       <c r="C18">
         <v>5.2</v>
       </c>
@@ -1971,13 +2339,13 @@
       <c r="E18" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="32"/>
-      <c r="H18" s="32"/>
-      <c r="I18" s="32"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="31"/>
     </row>
     <row r="19" spans="1:9" ht="86.4">
-      <c r="A19" s="31"/>
-      <c r="B19" s="31">
+      <c r="A19" s="33"/>
+      <c r="B19" s="33">
         <v>6</v>
       </c>
       <c r="C19">
@@ -1989,22 +2357,22 @@
       <c r="E19" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="F19" s="36">
+      <c r="F19" s="32">
         <v>46260</v>
       </c>
-      <c r="G19" s="32" t="s">
+      <c r="G19" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="H19" s="36">
+      <c r="H19" s="32">
         <v>46267</v>
       </c>
-      <c r="I19" s="32" t="s">
+      <c r="I19" s="31" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28.8">
-      <c r="A20" s="31"/>
-      <c r="B20" s="31"/>
+      <c r="A20" s="33"/>
+      <c r="B20" s="33"/>
       <c r="C20">
         <v>6.2</v>
       </c>
@@ -2014,14 +2382,14 @@
       <c r="E20" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
-      <c r="H20" s="32"/>
-      <c r="I20" s="32"/>
+      <c r="F20" s="31"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+      <c r="I20" s="31"/>
     </row>
     <row r="21" spans="1:9" ht="43.8" customHeight="1">
-      <c r="A21" s="31"/>
-      <c r="B21" s="31"/>
+      <c r="A21" s="33"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="18">
         <v>6.3</v>
       </c>
@@ -2031,14 +2399,14 @@
       <c r="E21" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="32"/>
-      <c r="I21" s="32"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+      <c r="I21" s="31"/>
     </row>
     <row r="22" spans="1:9" ht="28.8">
-      <c r="A22" s="31"/>
-      <c r="B22" s="31"/>
+      <c r="A22" s="33"/>
+      <c r="B22" s="33"/>
       <c r="C22">
         <v>6.4</v>
       </c>
@@ -2048,14 +2416,14 @@
       <c r="E22" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="32"/>
-      <c r="G22" s="32"/>
-      <c r="H22" s="32"/>
-      <c r="I22" s="32"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
     </row>
     <row r="23" spans="1:9" ht="28.8">
-      <c r="A23" s="31"/>
-      <c r="B23" s="31">
+      <c r="A23" s="33"/>
+      <c r="B23" s="33">
         <v>7</v>
       </c>
       <c r="C23">
@@ -2067,22 +2435,22 @@
       <c r="E23" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="36">
+      <c r="F23" s="32">
         <v>46260</v>
       </c>
-      <c r="G23" s="32" t="s">
+      <c r="G23" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="36">
+      <c r="H23" s="32">
         <v>46267</v>
       </c>
-      <c r="I23" s="32" t="s">
+      <c r="I23" s="31" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="31"/>
-      <c r="B24" s="31"/>
+      <c r="A24" s="33"/>
+      <c r="B24" s="33"/>
       <c r="C24">
         <v>7.2</v>
       </c>
@@ -2092,14 +2460,14 @@
       <c r="E24" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="F24" s="32"/>
-      <c r="G24" s="32"/>
-      <c r="H24" s="32"/>
-      <c r="I24" s="32"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
     </row>
     <row r="25" spans="1:9" ht="43.2">
-      <c r="A25" s="31"/>
-      <c r="B25" s="31">
+      <c r="A25" s="33"/>
+      <c r="B25" s="33">
         <v>8</v>
       </c>
       <c r="C25">
@@ -2111,22 +2479,22 @@
       <c r="E25" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="37">
+      <c r="F25" s="34">
         <v>46260</v>
       </c>
-      <c r="G25" s="32" t="s">
+      <c r="G25" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="H25" s="36">
+      <c r="H25" s="32">
         <v>46267</v>
       </c>
-      <c r="I25" s="32" t="s">
+      <c r="I25" s="31" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="28.8">
-      <c r="A26" s="31"/>
-      <c r="B26" s="31"/>
+      <c r="A26" s="33"/>
+      <c r="B26" s="33"/>
       <c r="C26">
         <v>8.1999999999999993</v>
       </c>
@@ -2136,10 +2504,10 @@
       <c r="E26" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="37"/>
-      <c r="G26" s="32"/>
-      <c r="H26" s="32"/>
-      <c r="I26" s="32"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="24"/>
@@ -2159,10 +2527,10 @@
       <c r="I27" s="23"/>
     </row>
     <row r="28" spans="1:9" ht="43.2">
-      <c r="A28" s="31">
+      <c r="A28" s="33">
         <v>3</v>
       </c>
-      <c r="B28" s="31">
+      <c r="B28" s="33">
         <v>9</v>
       </c>
       <c r="C28">
@@ -2174,22 +2542,22 @@
       <c r="E28" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="F28" s="36">
+      <c r="F28" s="32">
         <v>46268</v>
       </c>
-      <c r="G28" s="32" t="s">
+      <c r="G28" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="36">
+      <c r="H28" s="32">
         <v>46275</v>
       </c>
-      <c r="I28" s="32" t="s">
+      <c r="I28" s="31" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="28.8">
-      <c r="A29" s="31"/>
-      <c r="B29" s="31"/>
+      <c r="A29" s="33"/>
+      <c r="B29" s="33"/>
       <c r="C29">
         <v>9.1999999999999993</v>
       </c>
@@ -2199,14 +2567,14 @@
       <c r="E29" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="F29" s="36"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="36"/>
-      <c r="I29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="31"/>
     </row>
     <row r="30" spans="1:9" ht="28.8">
-      <c r="A30" s="31"/>
-      <c r="B30" s="31"/>
+      <c r="A30" s="33"/>
+      <c r="B30" s="33"/>
       <c r="C30">
         <v>9.3000000000000007</v>
       </c>
@@ -2216,50 +2584,17 @@
       <c r="E30" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F30" s="36"/>
-      <c r="G30" s="32"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="32"/>
+      <c r="I30" s="31"/>
     </row>
     <row r="31" spans="1:9">
-      <c r="A31" s="31"/>
-      <c r="B31" s="31"/>
+      <c r="A31" s="33"/>
+      <c r="B31" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="G19:G22"/>
-    <mergeCell ref="H19:H22"/>
-    <mergeCell ref="I28:I30"/>
-    <mergeCell ref="A3:A15"/>
-    <mergeCell ref="A17:A26"/>
-    <mergeCell ref="A28:A31"/>
-    <mergeCell ref="F28:F30"/>
-    <mergeCell ref="H28:H30"/>
-    <mergeCell ref="G28:G30"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="I19:I22"/>
-    <mergeCell ref="F3:F7"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F15:H15"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="J3:J15"/>
-    <mergeCell ref="H3:H7"/>
-    <mergeCell ref="F8:F11"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="I3:I7"/>
-    <mergeCell ref="G3:G7"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
     <mergeCell ref="F19:F22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="B25:B26"/>
@@ -2270,8 +2605,613 @@
     <mergeCell ref="B13:B14"/>
     <mergeCell ref="B17:B18"/>
     <mergeCell ref="B19:B22"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="J3:J15"/>
+    <mergeCell ref="H3:H7"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="I3:I7"/>
+    <mergeCell ref="G3:G7"/>
+    <mergeCell ref="A3:A15"/>
+    <mergeCell ref="A17:A26"/>
+    <mergeCell ref="A28:A31"/>
+    <mergeCell ref="F28:F30"/>
+    <mergeCell ref="H28:H30"/>
+    <mergeCell ref="G28:G30"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
+    <mergeCell ref="F3:F7"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="G19:G22"/>
+    <mergeCell ref="H19:H22"/>
+    <mergeCell ref="I28:I30"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="I19:I22"/>
+    <mergeCell ref="H17:H18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B077794A-BDEC-4305-8F7F-332456871660}">
+  <dimension ref="A1:K36"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12.44140625" customWidth="1"/>
+    <col min="2" max="2" width="63.77734375" customWidth="1"/>
+    <col min="4" max="5" width="10.88671875" customWidth="1"/>
+    <col min="6" max="6" width="38" style="40" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.109375" style="39" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.44140625" customWidth="1"/>
+    <col min="11" max="11" width="32.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="66" t="s">
+        <v>126</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+    </row>
+    <row r="2" spans="1:11" s="15" customFormat="1">
+      <c r="A2" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="B2" s="63" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="63" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="64" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="65" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="63" t="s">
+        <v>108</v>
+      </c>
+      <c r="I2" s="63" t="s">
+        <v>70</v>
+      </c>
+      <c r="J2" s="63" t="s">
+        <v>86</v>
+      </c>
+      <c r="K2" s="63" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="43.2" customHeight="1">
+      <c r="A3" s="33">
+        <v>1</v>
+      </c>
+      <c r="B3" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" s="33">
+        <v>8</v>
+      </c>
+      <c r="E3" s="35">
+        <v>46254</v>
+      </c>
+      <c r="F3" s="33" t="s">
+        <v>110</v>
+      </c>
+      <c r="G3" s="48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="28.8">
+      <c r="A4" s="33"/>
+      <c r="B4" s="38"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="33"/>
+      <c r="G4" s="48" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="72">
+      <c r="A5" s="33"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="33"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="33"/>
+      <c r="G5" s="48" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="33"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="33"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" s="48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="33"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="48" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="28.8">
+      <c r="A8" s="33"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G8" s="52" t="s">
+        <v>121</v>
+      </c>
+      <c r="K8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="43"/>
+      <c r="B9" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="45"/>
+      <c r="D9" s="45"/>
+      <c r="E9" s="47">
+        <v>46261</v>
+      </c>
+      <c r="F9" s="45"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="46"/>
+      <c r="I9" s="46"/>
+      <c r="J9" s="46"/>
+      <c r="K9" s="46"/>
+    </row>
+    <row r="10" spans="1:11" ht="57.6" customHeight="1">
+      <c r="A10" s="42">
+        <v>2</v>
+      </c>
+      <c r="B10" s="38" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="D10" s="33">
+        <v>8</v>
+      </c>
+      <c r="E10" s="35">
+        <v>46261</v>
+      </c>
+      <c r="F10" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="54" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="43.2">
+      <c r="A11" s="42"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="33"/>
+      <c r="G11" s="48" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
+      <c r="A12" s="42"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="48" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="28.8">
+      <c r="A13" s="42"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="33"/>
+      <c r="G13" s="48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="57.6">
+      <c r="A14" s="42"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="48" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="42"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="G15" s="48" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="42"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="52" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="57.6">
+      <c r="A17" s="42"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="G17" s="48" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" s="15" customFormat="1">
+      <c r="A18" s="57"/>
+      <c r="B18" s="58" t="s">
+        <v>119</v>
+      </c>
+      <c r="C18" s="57"/>
+      <c r="D18" s="57"/>
+      <c r="E18" s="59">
+        <v>46268</v>
+      </c>
+      <c r="F18" s="57" t="s">
+        <v>132</v>
+      </c>
+      <c r="G18" s="60"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="61"/>
+      <c r="K18" s="61"/>
+    </row>
+    <row r="19" spans="1:11" ht="86.4">
+      <c r="A19" s="33">
+        <v>3</v>
+      </c>
+      <c r="B19" s="41" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="D19" s="33">
+        <v>5</v>
+      </c>
+      <c r="E19" s="35">
+        <v>46268</v>
+      </c>
+      <c r="F19" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="G19" s="54" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="43.2">
+      <c r="A20" s="33"/>
+      <c r="B20" s="41"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="48" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="129.6">
+      <c r="A21" s="33"/>
+      <c r="B21" s="41"/>
+      <c r="C21" s="33"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="33" t="s">
+        <v>37</v>
+      </c>
+      <c r="G21" s="48" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="33"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="33"/>
+      <c r="G22" s="48" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="33"/>
+      <c r="B23" s="41"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="33"/>
+      <c r="G23" s="49" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="28.8">
+      <c r="A24" s="33"/>
+      <c r="B24" s="41"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="52" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11">
+      <c r="A25" s="43"/>
+      <c r="B25" s="44" t="s">
+        <v>118</v>
+      </c>
+      <c r="C25" s="45"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="47">
+        <v>46275</v>
+      </c>
+      <c r="F25" s="45"/>
+      <c r="G25" s="56"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="46"/>
+      <c r="J25" s="46"/>
+      <c r="K25" s="46"/>
+    </row>
+    <row r="26" spans="1:11" ht="43.2" customHeight="1">
+      <c r="A26" s="33">
+        <v>4</v>
+      </c>
+      <c r="B26" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="C26" s="33" t="s">
+        <v>109</v>
+      </c>
+      <c r="D26" s="33">
+        <v>8</v>
+      </c>
+      <c r="E26" s="35">
+        <v>46275</v>
+      </c>
+      <c r="F26" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="G26" s="53" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11">
+      <c r="A27" s="33"/>
+      <c r="B27" s="41"/>
+      <c r="C27" s="33"/>
+      <c r="D27" s="33"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="50" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="43.2">
+      <c r="A28" s="33"/>
+      <c r="B28" s="41"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="33" t="s">
+        <v>117</v>
+      </c>
+      <c r="G28" s="50" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="28.8">
+      <c r="A29" s="33"/>
+      <c r="B29" s="41"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="33"/>
+      <c r="G29" s="50" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="43.2">
+      <c r="A30" s="33"/>
+      <c r="B30" s="41"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="33"/>
+      <c r="E30" s="35"/>
+      <c r="F30" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="G30" s="50" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="28.8">
+      <c r="A31" s="33"/>
+      <c r="B31" s="41"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="33"/>
+      <c r="G31" s="50" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11">
+      <c r="A32" s="33"/>
+      <c r="B32" s="41"/>
+      <c r="C32" s="33"/>
+      <c r="D32" s="33"/>
+      <c r="E32" s="35"/>
+      <c r="F32" s="33"/>
+      <c r="G32" s="50" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
+      <c r="A33" s="33"/>
+      <c r="B33" s="41"/>
+      <c r="C33" s="33"/>
+      <c r="D33" s="33"/>
+      <c r="E33" s="35"/>
+      <c r="F33" s="33"/>
+      <c r="G33" s="50" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11">
+      <c r="A34" s="33"/>
+      <c r="B34" s="41"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="33"/>
+      <c r="E34" s="35"/>
+      <c r="F34" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="G34" s="50" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="28.8">
+      <c r="A35" s="33"/>
+      <c r="B35" s="41"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="35"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="51" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" s="15" customFormat="1">
+      <c r="A36" s="57"/>
+      <c r="B36" s="58" t="s">
+        <v>119</v>
+      </c>
+      <c r="C36" s="57"/>
+      <c r="D36" s="57"/>
+      <c r="E36" s="59">
+        <v>46282</v>
+      </c>
+      <c r="F36" s="57" t="s">
+        <v>131</v>
+      </c>
+      <c r="G36" s="62"/>
+      <c r="H36" s="61"/>
+      <c r="I36" s="61"/>
+      <c r="J36" s="61"/>
+      <c r="K36" s="61"/>
+    </row>
+  </sheetData>
+  <mergeCells count="31">
+    <mergeCell ref="E3:E8"/>
+    <mergeCell ref="E19:E24"/>
+    <mergeCell ref="E26:E35"/>
+    <mergeCell ref="E10:E17"/>
+    <mergeCell ref="D10:D17"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A3:A8"/>
+    <mergeCell ref="B3:B8"/>
+    <mergeCell ref="C3:C8"/>
+    <mergeCell ref="D3:D8"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="D26:D35"/>
+    <mergeCell ref="C26:C35"/>
+    <mergeCell ref="B26:B35"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="F28:F29"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="A26:A35"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="F21:F24"/>
+    <mergeCell ref="D19:D24"/>
+    <mergeCell ref="C19:C24"/>
+    <mergeCell ref="B19:B24"/>
+    <mergeCell ref="A19:A24"/>
+    <mergeCell ref="F10:F14"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="C10:C17"/>
+    <mergeCell ref="B10:B17"/>
+    <mergeCell ref="A10:A17"/>
+    <mergeCell ref="F3:F5"/>
+    <mergeCell ref="F6:F7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated product backlog; wireframes addition & estimation pending
</commit_message>
<xml_diff>
--- a/project_plan.xlsx
+++ b/project_plan.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41AF736-7A6A-4AF4-9A10-88AD80BDA3AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{228B6D37-7B31-4E3F-9D51-F31DB87662ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Plan" sheetId="1" r:id="rId1"/>
@@ -31,8 +31,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={233094A3-3D2A-436A-904F-A8273DA397F5}</author>
+    <author>tc={08942A35-04A9-4798-9BE7-511ACD0FC8D0}</author>
+  </authors>
+  <commentList>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{233094A3-3D2A-436A-904F-A8273DA397F5}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Should all skin concerns be listed when we are only addressing top n.</t>
+      </text>
+    </comment>
+    <comment ref="D7" authorId="1" shapeId="0" xr:uid="{08942A35-04A9-4798-9BE7-511ACD0FC8D0}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Upto what limit can a user repeat the process? </t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="171">
   <si>
     <t>Gain access to the Dev pannel of Shopify website for CelRevive from client.</t>
   </si>
@@ -837,7 +864,164 @@
     </r>
   </si>
   <si>
+    <t>Wireframe Reference</t>
+  </si>
+  <si>
+    <t>1. Blurry image should be rejected.
+2. A low lighting image should be rejected.
+3. A low resolution image should be rejected
+4. A combination of any/all of the above three should be rejected
+4. A proper image should not be rejected</t>
+  </si>
+  <si>
     <t>I can view my reccomendation page with the following fields:
+1. Hello "user_full_name"! 
+2. Skin analysis results : Primary Concerns : only those detected through selfie.</t>
+  </si>
+  <si>
+    <t>XS</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>XL</t>
+  </si>
+  <si>
+    <t>XXL</t>
+  </si>
+  <si>
+    <t>XXXL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSHIRT SIZING </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">press the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">add to cart 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">button </t>
+    </r>
+  </si>
+  <si>
+    <t>todo/wip/done - states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a </t>
+  </si>
+  <si>
+    <t>Difficulty</t>
+  </si>
+  <si>
+    <t>Scale : 1-5</t>
+  </si>
+  <si>
+    <t>Final Weightage</t>
+  </si>
+  <si>
+    <t>Ease</t>
+  </si>
+  <si>
+    <t>I can add the reccomended formulation to my shopping cart .</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Detected skin concerns should be from the series:
+SC0001 - SC0019 &amp; SC1001 - SC1009
+2. If no skin concern is detected (perfectly fit skin) then Skin analysis results should show the following message:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Your skin looks perfect!".
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3. If the image contains one or multiple particular skin concerns then, all of those should be shown in the Skin analysis results: Primary Concerns.
+4. No other skin concerns should be shown in the Skin analysis results: Primary Concerns other than the ones really existing in the images.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Detected skin concerns should be from the series:
+SC0001-SC0019 , SC1001-SC1009 &amp;
+SC2001-SC2004.
+2. If no skin concern is detected(perfectly fit skin) then Skin analysis results should show the following message:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">"Your skin looks perfect!"
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">3.If the image &amp; questionnaire contains one or multiple particular skin concerns then, all of those should be shown in the Skin analysis results: Primary Concerns.
+4.No other skins concerns should be shown in the Skin analysis results: Primary Concerns other than the ones really existing in the images and questionnaire.
+5. The total formulation must always weigh 100g total.
+6. The percentage of actives in formulation must be listed.
+7. The formulation explanation must correctly reflect the reason for choosing the actives and bases.
+8. Skin analysis result:Skin Type, Sensitive Level, Allergens: must exactly match the answers provided by the user via the questionnaire.
+9. The reccomended formula must not contain any harmful or unsuitable ingredients as per the answers provided by the user via the questionnaire.
+10. The actives and base comprising the reccomended formulation must be compatible with each other, and relevant to the user's skin concerns.
+11. The cost of actives and base comprising the reccomended formulation must be calculated with their accurate cost/g.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">I can view my reccomendation page with the following fields:
 1. Hello "user_full_name"! 
 2. Skin analysis results : Primary Concerns :  those detected through the combination of skin concerns from both image and questionnaire.
 3.Skin analysis results: Skin Type: detected through questionnaire answers.
@@ -846,128 +1030,91 @@
 6. Reccomended for you: Base :
 selected through questionnaire answers.
 7. Reccomended for you : Active Ingredients: those detected through selfie and questionnaire skin concerns.
-8. Reccomended for you: Why this formula: explained by LLM for selected actives detected through selfie and questionnaire skin concerns</t>
-  </si>
-  <si>
-    <t>Wireframe Reference</t>
-  </si>
-  <si>
-    <t>1. Blurry image should be rejected.
-2. A low lighting image should be rejected.
-3. A low resolution image should be rejected
-4. A combination of any/all of the above three should be rejected
-4. A proper image should not be rejected</t>
-  </si>
-  <si>
-    <t>I can view my reccomendation page with the following fields:
-1. Hello "user_full_name"! 
-2. Skin analysis results : Primary Concerns : only those detected through selfie.</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Detected skin concerns should be from the series:
-SC0001 - SC0019 &amp; SC1001 - SC1009
-2. If no skin concern is detected (perfectly fit skin) then Skin analysis results should show the following message:
+8. Reccomended for you: Why this formula: explained by LLM for selected actives detected through selfie and questionnaire skin concerns
+9.Reccomended for you: Cost: Total cost of the reccomended formulation. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[add in wireframes]</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">I can repeat my AI skin analysis. </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1.Upon </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">add to cart </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>button being clicked, the reccomended formulation along with cost , should be saved for the user and added to their shopping cart, allowing them to buy later at their convenience. 
+2. The saved formulation in [1] must exactly match the reccomended formulation.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">press the 
 </t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">"Your skin looks perfect!".
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">[repeat reccomendation process] 
 </t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3. If the image contains one or multiple particular skin concerns that should all be shown in the Skin analysis results: Primary Concerns.
-4. No other skin concerns should be shown in the Skin analysis results: Primary Concerns other than the ones really existing in the images.</t>
-    </r>
-  </si>
-  <si>
-    <t>XS</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>M</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>XL</t>
-  </si>
-  <si>
-    <t>XXL</t>
-  </si>
-  <si>
-    <t>XXXL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TSHIRT SIZING </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">press the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">add to cart 
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">button
 </t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">button </t>
-    </r>
-  </si>
-  <si>
-    <t>todo/wip/done - states</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a </t>
-  </si>
-  <si>
-    <t>Difficulty</t>
-  </si>
-  <si>
-    <t>Scale : 1-5</t>
-  </si>
-  <si>
-    <t>Final Weightage</t>
-  </si>
-  <si>
-    <t>Ease</t>
+  </si>
+  <si>
+    <t>Sprint Id</t>
+  </si>
+  <si>
+    <t>Story Point</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1002,6 +1149,20 @@
       <name val="Arial Unicode MS"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFC00000"/>
       <name val="Calibri"/>
@@ -1156,7 +1317,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1310,30 +1471,6 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1343,8 +1480,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1353,13 +1490,50 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1375,6 +1549,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1662,6 +1840,17 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="E5" dT="2026-08-20T15:41:46.67" personId="{00000000-0000-0000-0000-000000000000}" id="{233094A3-3D2A-436A-904F-A8273DA397F5}">
+    <text>Should all skin concerns be listed when we are only addressing top n.</text>
+  </threadedComment>
+  <threadedComment ref="D7" dT="2026-08-20T15:38:33.80" personId="{00000000-0000-0000-0000-000000000000}" id="{08942A35-04A9-4798-9BE7-511ACD0FC8D0}">
+    <text xml:space="preserve">Upto what limit can a user repeat the process? </text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G25"/>
@@ -2149,20 +2338,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="62"/>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
-      <c r="G1" s="62"/>
-      <c r="H1" s="62"/>
-      <c r="I1" s="62"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="15" t="s">
@@ -2203,10 +2392,10 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="58.8" customHeight="1">
-      <c r="A3" s="58">
+      <c r="A3" s="71">
         <v>1</v>
       </c>
-      <c r="B3" s="58">
+      <c r="B3" s="71">
         <v>1</v>
       </c>
       <c r="C3">
@@ -2218,25 +2407,25 @@
       <c r="E3" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="F3" s="57">
+      <c r="F3" s="74">
         <v>46252</v>
       </c>
-      <c r="G3" s="58" t="s">
+      <c r="G3" s="71" t="s">
         <v>94</v>
       </c>
-      <c r="H3" s="57">
+      <c r="H3" s="74">
         <v>46259</v>
       </c>
-      <c r="I3" s="58" t="s">
+      <c r="I3" s="71" t="s">
         <v>88</v>
       </c>
-      <c r="J3" s="58" t="s">
+      <c r="J3" s="71" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="54.6" customHeight="1">
-      <c r="A4" s="58"/>
-      <c r="B4" s="58"/>
+      <c r="A4" s="71"/>
+      <c r="B4" s="71"/>
       <c r="C4">
         <v>1.2</v>
       </c>
@@ -2246,15 +2435,15 @@
       <c r="E4" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="57"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
-      <c r="I4" s="58"/>
-      <c r="J4" s="58"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="71"/>
+      <c r="H4" s="71"/>
+      <c r="I4" s="71"/>
+      <c r="J4" s="71"/>
     </row>
     <row r="5" spans="1:12" ht="33.6" customHeight="1">
-      <c r="A5" s="58"/>
-      <c r="B5" s="58"/>
+      <c r="A5" s="71"/>
+      <c r="B5" s="71"/>
       <c r="C5">
         <v>1.3</v>
       </c>
@@ -2264,15 +2453,15 @@
       <c r="E5" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="57"/>
-      <c r="G5" s="58"/>
-      <c r="H5" s="58"/>
-      <c r="I5" s="58"/>
-      <c r="J5" s="58"/>
+      <c r="F5" s="74"/>
+      <c r="G5" s="71"/>
+      <c r="H5" s="71"/>
+      <c r="I5" s="71"/>
+      <c r="J5" s="71"/>
     </row>
     <row r="6" spans="1:12" ht="26.4" customHeight="1">
-      <c r="A6" s="58"/>
-      <c r="B6" s="58"/>
+      <c r="A6" s="71"/>
+      <c r="B6" s="71"/>
       <c r="C6">
         <v>1.4</v>
       </c>
@@ -2282,15 +2471,15 @@
       <c r="E6" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="57"/>
-      <c r="G6" s="58"/>
-      <c r="H6" s="58"/>
-      <c r="I6" s="58"/>
-      <c r="J6" s="58"/>
+      <c r="F6" s="74"/>
+      <c r="G6" s="71"/>
+      <c r="H6" s="71"/>
+      <c r="I6" s="71"/>
+      <c r="J6" s="71"/>
     </row>
     <row r="7" spans="1:12" ht="72.599999999999994" customHeight="1">
-      <c r="A7" s="58"/>
-      <c r="B7" s="58"/>
+      <c r="A7" s="71"/>
+      <c r="B7" s="71"/>
       <c r="C7">
         <v>1.5</v>
       </c>
@@ -2300,15 +2489,15 @@
       <c r="E7" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="F7" s="57"/>
-      <c r="G7" s="58"/>
-      <c r="H7" s="58"/>
-      <c r="I7" s="58"/>
-      <c r="J7" s="58"/>
+      <c r="F7" s="74"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="71"/>
+      <c r="J7" s="71"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="58"/>
-      <c r="B8" s="58">
+      <c r="A8" s="71"/>
+      <c r="B8" s="71">
         <v>2</v>
       </c>
       <c r="C8">
@@ -2320,23 +2509,23 @@
       <c r="E8" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="57">
+      <c r="F8" s="74">
         <v>46252</v>
       </c>
-      <c r="G8" s="58" t="s">
+      <c r="G8" s="71" t="s">
         <v>90</v>
       </c>
-      <c r="H8" s="57">
+      <c r="H8" s="74">
         <v>46258</v>
       </c>
-      <c r="I8" s="58" t="s">
+      <c r="I8" s="71" t="s">
         <v>89</v>
       </c>
-      <c r="J8" s="58"/>
+      <c r="J8" s="71"/>
     </row>
     <row r="9" spans="1:12" ht="28.8">
-      <c r="A9" s="58"/>
-      <c r="B9" s="58"/>
+      <c r="A9" s="71"/>
+      <c r="B9" s="71"/>
       <c r="C9">
         <v>2.2000000000000002</v>
       </c>
@@ -2346,15 +2535,15 @@
       <c r="E9" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="57"/>
-      <c r="G9" s="58"/>
-      <c r="H9" s="57"/>
-      <c r="I9" s="58"/>
-      <c r="J9" s="58"/>
+      <c r="F9" s="74"/>
+      <c r="G9" s="71"/>
+      <c r="H9" s="74"/>
+      <c r="I9" s="71"/>
+      <c r="J9" s="71"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
-      <c r="A10" s="58"/>
-      <c r="B10" s="58"/>
+      <c r="A10" s="71"/>
+      <c r="B10" s="71"/>
       <c r="C10">
         <v>2.2999999999999998</v>
       </c>
@@ -2364,15 +2553,15 @@
       <c r="E10" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="57"/>
-      <c r="G10" s="58"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="58"/>
-      <c r="J10" s="58"/>
+      <c r="F10" s="74"/>
+      <c r="G10" s="71"/>
+      <c r="H10" s="74"/>
+      <c r="I10" s="71"/>
+      <c r="J10" s="71"/>
     </row>
     <row r="11" spans="1:12" ht="28.8">
-      <c r="A11" s="58"/>
-      <c r="B11" s="58">
+      <c r="A11" s="71"/>
+      <c r="B11" s="71">
         <v>3</v>
       </c>
       <c r="C11">
@@ -2384,15 +2573,15 @@
       <c r="E11" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="F11" s="57"/>
-      <c r="G11" s="58"/>
-      <c r="H11" s="57"/>
-      <c r="I11" s="58"/>
-      <c r="J11" s="58"/>
+      <c r="F11" s="74"/>
+      <c r="G11" s="71"/>
+      <c r="H11" s="74"/>
+      <c r="I11" s="71"/>
+      <c r="J11" s="71"/>
     </row>
     <row r="12" spans="1:12" ht="28.8">
-      <c r="A12" s="58"/>
-      <c r="B12" s="58"/>
+      <c r="A12" s="71"/>
+      <c r="B12" s="71"/>
       <c r="C12">
         <v>3.2</v>
       </c>
@@ -2414,11 +2603,11 @@
       <c r="I12" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="J12" s="58"/>
+      <c r="J12" s="71"/>
     </row>
     <row r="13" spans="1:12" ht="28.8">
-      <c r="A13" s="58"/>
-      <c r="B13" s="58">
+      <c r="A13" s="71"/>
+      <c r="B13" s="71">
         <v>4</v>
       </c>
       <c r="C13">
@@ -2442,11 +2631,11 @@
       <c r="I13" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="J13" s="58"/>
+      <c r="J13" s="71"/>
     </row>
     <row r="14" spans="1:12" ht="28.8">
-      <c r="A14" s="58"/>
-      <c r="B14" s="58"/>
+      <c r="A14" s="71"/>
+      <c r="B14" s="71"/>
       <c r="C14">
         <v>4.2</v>
       </c>
@@ -2468,10 +2657,10 @@
       <c r="I14" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="J14" s="58"/>
+      <c r="J14" s="71"/>
     </row>
     <row r="15" spans="1:12" ht="28.8">
-      <c r="A15" s="58"/>
+      <c r="A15" s="71"/>
       <c r="B15" s="14">
         <v>9</v>
       </c>
@@ -2484,15 +2673,15 @@
       <c r="E15" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F15" s="57" t="s">
+      <c r="F15" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="G15" s="57"/>
-      <c r="H15" s="57"/>
+      <c r="G15" s="74"/>
+      <c r="H15" s="74"/>
       <c r="I15" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="J15" s="58"/>
+      <c r="J15" s="71"/>
       <c r="L15" t="s">
         <v>98</v>
       </c>
@@ -2501,10 +2690,10 @@
       <c r="A16" s="23"/>
       <c r="B16" s="24"/>
       <c r="C16" s="25"/>
-      <c r="D16" s="64" t="s">
+      <c r="D16" s="75" t="s">
         <v>95</v>
       </c>
-      <c r="E16" s="64"/>
+      <c r="E16" s="75"/>
       <c r="F16" s="26">
         <v>46198</v>
       </c>
@@ -2515,10 +2704,10 @@
       <c r="I16" s="24"/>
     </row>
     <row r="17" spans="1:9" ht="86.4">
-      <c r="A17" s="58">
+      <c r="A17" s="71">
         <v>2</v>
       </c>
-      <c r="B17" s="58">
+      <c r="B17" s="71">
         <v>5</v>
       </c>
       <c r="C17">
@@ -2533,19 +2722,19 @@
       <c r="F17" s="21">
         <v>46260</v>
       </c>
-      <c r="G17" s="61" t="s">
+      <c r="G17" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="H17" s="60">
+      <c r="H17" s="70">
         <v>46262</v>
       </c>
-      <c r="I17" s="61" t="s">
+      <c r="I17" s="69" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="28.8">
-      <c r="A18" s="58"/>
-      <c r="B18" s="58"/>
+      <c r="A18" s="71"/>
+      <c r="B18" s="71"/>
       <c r="C18">
         <v>5.2</v>
       </c>
@@ -2555,13 +2744,13 @@
       <c r="E18" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
-      <c r="I18" s="61"/>
+      <c r="G18" s="69"/>
+      <c r="H18" s="69"/>
+      <c r="I18" s="69"/>
     </row>
     <row r="19" spans="1:9" ht="86.4">
-      <c r="A19" s="58"/>
-      <c r="B19" s="58">
+      <c r="A19" s="71"/>
+      <c r="B19" s="71">
         <v>6</v>
       </c>
       <c r="C19">
@@ -2573,22 +2762,22 @@
       <c r="E19" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="F19" s="60">
+      <c r="F19" s="70">
         <v>46260</v>
       </c>
-      <c r="G19" s="61" t="s">
+      <c r="G19" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="H19" s="60">
+      <c r="H19" s="70">
         <v>46267</v>
       </c>
-      <c r="I19" s="61" t="s">
+      <c r="I19" s="69" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="28.8">
-      <c r="A20" s="58"/>
-      <c r="B20" s="58"/>
+      <c r="A20" s="71"/>
+      <c r="B20" s="71"/>
       <c r="C20">
         <v>6.2</v>
       </c>
@@ -2598,14 +2787,14 @@
       <c r="E20" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="F20" s="61"/>
-      <c r="G20" s="61"/>
-      <c r="H20" s="61"/>
-      <c r="I20" s="61"/>
+      <c r="F20" s="69"/>
+      <c r="G20" s="69"/>
+      <c r="H20" s="69"/>
+      <c r="I20" s="69"/>
     </row>
     <row r="21" spans="1:9" ht="43.8" customHeight="1">
-      <c r="A21" s="58"/>
-      <c r="B21" s="58"/>
+      <c r="A21" s="71"/>
+      <c r="B21" s="71"/>
       <c r="C21" s="18">
         <v>6.3</v>
       </c>
@@ -2615,14 +2804,14 @@
       <c r="E21" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F21" s="61"/>
-      <c r="G21" s="61"/>
-      <c r="H21" s="61"/>
-      <c r="I21" s="61"/>
+      <c r="F21" s="69"/>
+      <c r="G21" s="69"/>
+      <c r="H21" s="69"/>
+      <c r="I21" s="69"/>
     </row>
     <row r="22" spans="1:9" ht="28.8">
-      <c r="A22" s="58"/>
-      <c r="B22" s="58"/>
+      <c r="A22" s="71"/>
+      <c r="B22" s="71"/>
       <c r="C22">
         <v>6.4</v>
       </c>
@@ -2632,14 +2821,14 @@
       <c r="E22" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="F22" s="61"/>
-      <c r="G22" s="61"/>
-      <c r="H22" s="61"/>
-      <c r="I22" s="61"/>
+      <c r="F22" s="69"/>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
+      <c r="I22" s="69"/>
     </row>
     <row r="23" spans="1:9" ht="28.8">
-      <c r="A23" s="58"/>
-      <c r="B23" s="58">
+      <c r="A23" s="71"/>
+      <c r="B23" s="71">
         <v>7</v>
       </c>
       <c r="C23">
@@ -2651,22 +2840,22 @@
       <c r="E23" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="F23" s="60">
+      <c r="F23" s="70">
         <v>46260</v>
       </c>
-      <c r="G23" s="61" t="s">
+      <c r="G23" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="60">
+      <c r="H23" s="70">
         <v>46267</v>
       </c>
-      <c r="I23" s="61" t="s">
+      <c r="I23" s="69" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="58"/>
-      <c r="B24" s="58"/>
+      <c r="A24" s="71"/>
+      <c r="B24" s="71"/>
       <c r="C24">
         <v>7.2</v>
       </c>
@@ -2676,14 +2865,14 @@
       <c r="E24" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="F24" s="61"/>
-      <c r="G24" s="61"/>
-      <c r="H24" s="61"/>
-      <c r="I24" s="61"/>
+      <c r="F24" s="69"/>
+      <c r="G24" s="69"/>
+      <c r="H24" s="69"/>
+      <c r="I24" s="69"/>
     </row>
     <row r="25" spans="1:9" ht="43.2">
-      <c r="A25" s="58"/>
-      <c r="B25" s="58">
+      <c r="A25" s="71"/>
+      <c r="B25" s="71">
         <v>8</v>
       </c>
       <c r="C25">
@@ -2695,22 +2884,22 @@
       <c r="E25" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="63">
+      <c r="F25" s="72">
         <v>46260</v>
       </c>
-      <c r="G25" s="61" t="s">
+      <c r="G25" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="H25" s="60">
+      <c r="H25" s="70">
         <v>46267</v>
       </c>
-      <c r="I25" s="61" t="s">
+      <c r="I25" s="69" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="28.8">
-      <c r="A26" s="58"/>
-      <c r="B26" s="58"/>
+      <c r="A26" s="71"/>
+      <c r="B26" s="71"/>
       <c r="C26">
         <v>8.1999999999999993</v>
       </c>
@@ -2720,10 +2909,10 @@
       <c r="E26" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="F26" s="63"/>
-      <c r="G26" s="61"/>
-      <c r="H26" s="61"/>
-      <c r="I26" s="61"/>
+      <c r="F26" s="72"/>
+      <c r="G26" s="69"/>
+      <c r="H26" s="69"/>
+      <c r="I26" s="69"/>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="24"/>
@@ -2743,10 +2932,10 @@
       <c r="I27" s="23"/>
     </row>
     <row r="28" spans="1:9" ht="43.2">
-      <c r="A28" s="58">
+      <c r="A28" s="71">
         <v>3</v>
       </c>
-      <c r="B28" s="58">
+      <c r="B28" s="71">
         <v>9</v>
       </c>
       <c r="C28">
@@ -2758,22 +2947,22 @@
       <c r="E28" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="F28" s="60">
+      <c r="F28" s="70">
         <v>46268</v>
       </c>
-      <c r="G28" s="61" t="s">
+      <c r="G28" s="69" t="s">
         <v>94</v>
       </c>
-      <c r="H28" s="60">
+      <c r="H28" s="70">
         <v>46275</v>
       </c>
-      <c r="I28" s="61" t="s">
+      <c r="I28" s="69" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="28.8">
-      <c r="A29" s="58"/>
-      <c r="B29" s="58"/>
+      <c r="A29" s="71"/>
+      <c r="B29" s="71"/>
       <c r="C29">
         <v>9.1999999999999993</v>
       </c>
@@ -2783,14 +2972,14 @@
       <c r="E29" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="F29" s="60"/>
-      <c r="G29" s="61"/>
-      <c r="H29" s="60"/>
-      <c r="I29" s="61"/>
+      <c r="F29" s="70"/>
+      <c r="G29" s="69"/>
+      <c r="H29" s="70"/>
+      <c r="I29" s="69"/>
     </row>
     <row r="30" spans="1:9" ht="28.8">
-      <c r="A30" s="58"/>
-      <c r="B30" s="58"/>
+      <c r="A30" s="71"/>
+      <c r="B30" s="71"/>
       <c r="C30">
         <v>9.3000000000000007</v>
       </c>
@@ -2800,25 +2989,36 @@
       <c r="E30" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F30" s="60"/>
-      <c r="G30" s="61"/>
-      <c r="H30" s="60"/>
-      <c r="I30" s="61"/>
+      <c r="F30" s="70"/>
+      <c r="G30" s="69"/>
+      <c r="H30" s="70"/>
+      <c r="I30" s="69"/>
     </row>
     <row r="31" spans="1:9">
-      <c r="A31" s="58"/>
-      <c r="B31" s="58"/>
+      <c r="A31" s="71"/>
+      <c r="B31" s="71"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="G19:G22"/>
-    <mergeCell ref="H19:H22"/>
-    <mergeCell ref="I28:I30"/>
-    <mergeCell ref="I23:I24"/>
-    <mergeCell ref="I19:I22"/>
-    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B22"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="J3:J15"/>
+    <mergeCell ref="H3:H7"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="I3:I7"/>
+    <mergeCell ref="G3:G7"/>
+    <mergeCell ref="A3:A15"/>
+    <mergeCell ref="F3:F7"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="B13:B14"/>
     <mergeCell ref="A17:A26"/>
     <mergeCell ref="A28:A31"/>
     <mergeCell ref="F28:F30"/>
@@ -2831,29 +3031,18 @@
     <mergeCell ref="G25:G26"/>
     <mergeCell ref="H25:H26"/>
     <mergeCell ref="G17:G18"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="J3:J15"/>
-    <mergeCell ref="H3:H7"/>
-    <mergeCell ref="F8:F11"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="I3:I7"/>
-    <mergeCell ref="G3:G7"/>
-    <mergeCell ref="A3:A15"/>
-    <mergeCell ref="F3:F7"/>
-    <mergeCell ref="F15:H15"/>
     <mergeCell ref="F19:F22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="B28:B31"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B19:B22"/>
-    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="G19:G22"/>
+    <mergeCell ref="H19:H22"/>
+    <mergeCell ref="I28:I30"/>
+    <mergeCell ref="I23:I24"/>
+    <mergeCell ref="I19:I22"/>
+    <mergeCell ref="H17:H18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2862,7 +3051,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B077794A-BDEC-4305-8F7F-332456871660}">
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:V42"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.44140625" customWidth="1"/>
@@ -2877,43 +3066,44 @@
     <col min="11" max="11" width="7.44140625" customWidth="1"/>
     <col min="13" max="13" width="32.77734375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
-      <c r="A1" s="68" t="s">
+    <row r="1" spans="1:22">
+      <c r="A1" s="60" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="68"/>
-      <c r="C1" s="68"/>
-      <c r="D1" s="69"/>
-      <c r="E1" s="69"/>
-      <c r="F1" s="69"/>
-      <c r="G1" s="69"/>
-      <c r="H1" s="69"/>
-      <c r="I1" s="69"/>
-      <c r="J1" s="69"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-    </row>
-    <row r="2" spans="1:14">
-      <c r="A2" s="68"/>
-      <c r="B2" s="59" t="s">
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
+    </row>
+    <row r="2" spans="1:22">
+      <c r="A2" s="60"/>
+      <c r="B2" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
-      <c r="L2" s="69"/>
-      <c r="M2" s="69"/>
-    </row>
-    <row r="3" spans="1:14" s="15" customFormat="1" ht="16.2" customHeight="1">
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
+    </row>
+    <row r="3" spans="1:22" s="15" customFormat="1" ht="16.2" customHeight="1">
       <c r="A3" s="53" t="s">
         <v>104</v>
       </c>
@@ -2954,59 +3144,77 @@
         <v>97</v>
       </c>
       <c r="N3" s="15" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" ht="43.2">
+        <v>156</v>
+      </c>
+      <c r="Q3" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="R3" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="S3" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="T3" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="U3" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="V3" s="15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="43.2">
       <c r="A4" s="33"/>
       <c r="B4" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="C4" s="66" t="s">
+      <c r="C4" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="D4" s="66" t="s">
+      <c r="D4" s="58" t="s">
         <v>137</v>
       </c>
       <c r="E4" s="39" t="s">
         <v>55</v>
       </c>
       <c r="F4" s="33"/>
-      <c r="G4" s="70"/>
+      <c r="G4" s="62"/>
       <c r="I4" s="39"/>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:22">
       <c r="A5" s="33"/>
       <c r="B5" s="14"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
       <c r="E5" s="39" t="s">
         <v>85</v>
       </c>
       <c r="F5" s="33"/>
-      <c r="G5" s="70"/>
+      <c r="G5" s="62"/>
       <c r="I5" s="39"/>
     </row>
-    <row r="6" spans="1:14" ht="42" customHeight="1">
+    <row r="6" spans="1:22" ht="42" customHeight="1">
       <c r="A6" s="33"/>
       <c r="B6" s="14"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
       <c r="E6" s="39" t="s">
         <v>87</v>
       </c>
       <c r="F6" s="33"/>
-      <c r="G6" s="70"/>
+      <c r="G6" s="62"/>
       <c r="I6" s="39"/>
     </row>
-    <row r="7" spans="1:14" ht="115.2">
+    <row r="7" spans="1:22" ht="115.2">
       <c r="A7" s="33">
         <v>1</v>
       </c>
       <c r="B7" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="C7" s="66" t="s">
+      <c r="C7" s="58" t="s">
         <v>139</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -3018,7 +3226,7 @@
       <c r="F7" s="33">
         <v>8</v>
       </c>
-      <c r="G7" s="70">
+      <c r="G7" s="62">
         <v>46254</v>
       </c>
       <c r="H7" s="33" t="s">
@@ -3026,7 +3234,7 @@
       </c>
       <c r="I7" s="39"/>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:22">
       <c r="A8" s="33"/>
       <c r="B8" s="14"/>
       <c r="C8" s="14"/>
@@ -3035,10 +3243,10 @@
         <v>85</v>
       </c>
       <c r="F8" s="33"/>
-      <c r="G8" s="70"/>
+      <c r="G8" s="62"/>
       <c r="I8" s="39"/>
     </row>
-    <row r="9" spans="1:14" ht="28.8">
+    <row r="9" spans="1:22" ht="28.8">
       <c r="A9" s="33"/>
       <c r="B9" s="14"/>
       <c r="C9" s="14"/>
@@ -3047,10 +3255,10 @@
         <v>87</v>
       </c>
       <c r="F9" s="33"/>
-      <c r="G9" s="70"/>
+      <c r="G9" s="62"/>
       <c r="I9" s="39"/>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:22">
       <c r="A10" s="33"/>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -3059,7 +3267,7 @@
         <v>140</v>
       </c>
       <c r="F10" s="33"/>
-      <c r="G10" s="70"/>
+      <c r="G10" s="62"/>
       <c r="H10" s="33" t="s">
         <v>56</v>
       </c>
@@ -3067,26 +3275,26 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:22">
       <c r="A11" s="33"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="33"/>
-      <c r="G11" s="70"/>
+      <c r="G11" s="62"/>
       <c r="I11" s="39" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="28.8">
+    <row r="12" spans="1:22" ht="28.8">
       <c r="A12" s="33"/>
       <c r="B12" s="14"/>
       <c r="C12" s="14"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="33"/>
-      <c r="G12" s="70"/>
+      <c r="G12" s="62"/>
       <c r="H12" s="14" t="s">
         <v>118</v>
       </c>
@@ -3097,7 +3305,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:22">
       <c r="A13" s="14"/>
       <c r="B13" s="14"/>
       <c r="C13" s="14"/>
@@ -3107,11 +3315,11 @@
       <c r="H13" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="I13" s="65" t="s">
+      <c r="I13" s="57" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:22">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -3120,9 +3328,9 @@
       <c r="F14" s="14"/>
       <c r="G14" s="22"/>
       <c r="H14" s="14"/>
-      <c r="I14" s="65"/>
-    </row>
-    <row r="15" spans="1:14">
+      <c r="I14" s="57"/>
+    </row>
+    <row r="15" spans="1:22">
       <c r="A15" s="34"/>
       <c r="B15" s="34"/>
       <c r="C15" s="34"/>
@@ -3141,20 +3349,20 @@
       <c r="L15" s="37"/>
       <c r="M15" s="37"/>
     </row>
-    <row r="16" spans="1:14" ht="57.6" customHeight="1">
+    <row r="16" spans="1:22" ht="57.6" customHeight="1">
       <c r="A16" s="33">
         <v>2</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14"/>
-      <c r="D16" s="67" t="s">
+      <c r="D16" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="E16" s="67"/>
+      <c r="E16" s="59"/>
       <c r="F16" s="33">
         <v>8</v>
       </c>
-      <c r="G16" s="70">
+      <c r="G16" s="62">
         <v>46261</v>
       </c>
       <c r="H16" s="33" t="s">
@@ -3168,10 +3376,10 @@
       <c r="A17" s="33"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
-      <c r="D17" s="67"/>
-      <c r="E17" s="67"/>
+      <c r="D17" s="59"/>
+      <c r="E17" s="59"/>
       <c r="F17" s="33"/>
-      <c r="G17" s="70"/>
+      <c r="G17" s="62"/>
       <c r="I17" s="39" t="s">
         <v>50</v>
       </c>
@@ -3180,10 +3388,10 @@
       <c r="A18" s="33"/>
       <c r="B18" s="14"/>
       <c r="C18" s="14"/>
-      <c r="D18" s="67"/>
-      <c r="E18" s="67"/>
+      <c r="D18" s="59"/>
+      <c r="E18" s="59"/>
       <c r="F18" s="33"/>
-      <c r="G18" s="70"/>
+      <c r="G18" s="62"/>
       <c r="I18" s="39" t="s">
         <v>51</v>
       </c>
@@ -3192,10 +3400,10 @@
       <c r="A19" s="33"/>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
-      <c r="D19" s="67"/>
-      <c r="E19" s="67"/>
+      <c r="D19" s="59"/>
+      <c r="E19" s="59"/>
       <c r="F19" s="33"/>
-      <c r="G19" s="70"/>
+      <c r="G19" s="62"/>
       <c r="I19" s="39" t="s">
         <v>52</v>
       </c>
@@ -3204,10 +3412,10 @@
       <c r="A20" s="33"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
-      <c r="D20" s="67"/>
-      <c r="E20" s="67"/>
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
       <c r="F20" s="33"/>
-      <c r="G20" s="70"/>
+      <c r="G20" s="62"/>
       <c r="I20" s="39" t="s">
         <v>53</v>
       </c>
@@ -3216,10 +3424,10 @@
       <c r="A21" s="33"/>
       <c r="B21" s="14"/>
       <c r="C21" s="14"/>
-      <c r="D21" s="67"/>
-      <c r="E21" s="67"/>
+      <c r="D21" s="59"/>
+      <c r="E21" s="59"/>
       <c r="F21" s="33"/>
-      <c r="G21" s="70"/>
+      <c r="G21" s="62"/>
       <c r="H21" s="33" t="s">
         <v>110</v>
       </c>
@@ -3231,10 +3439,10 @@
       <c r="A22" s="33"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
-      <c r="D22" s="67"/>
-      <c r="E22" s="67"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="59"/>
       <c r="F22" s="33"/>
-      <c r="G22" s="70"/>
+      <c r="G22" s="62"/>
       <c r="I22" s="43" t="s">
         <v>57</v>
       </c>
@@ -3243,10 +3451,10 @@
       <c r="A23" s="33"/>
       <c r="B23" s="14"/>
       <c r="C23" s="14"/>
-      <c r="D23" s="67"/>
-      <c r="E23" s="67"/>
+      <c r="D23" s="59"/>
+      <c r="E23" s="59"/>
       <c r="F23" s="33"/>
-      <c r="G23" s="70"/>
+      <c r="G23" s="62"/>
       <c r="H23" s="14" t="s">
         <v>125</v>
       </c>
@@ -3281,14 +3489,14 @@
       </c>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
-      <c r="D25" s="67" t="s">
+      <c r="D25" s="59" t="s">
         <v>112</v>
       </c>
-      <c r="E25" s="67"/>
+      <c r="E25" s="59"/>
       <c r="F25" s="33">
         <v>5</v>
       </c>
-      <c r="G25" s="70">
+      <c r="G25" s="62">
         <v>46268</v>
       </c>
       <c r="H25" s="33" t="s">
@@ -3302,10 +3510,10 @@
       <c r="A26" s="33"/>
       <c r="B26" s="14"/>
       <c r="C26" s="14"/>
-      <c r="D26" s="67"/>
-      <c r="E26" s="67"/>
+      <c r="D26" s="59"/>
+      <c r="E26" s="59"/>
       <c r="F26" s="33"/>
-      <c r="G26" s="70"/>
+      <c r="G26" s="62"/>
       <c r="I26" s="39" t="s">
         <v>61</v>
       </c>
@@ -3314,10 +3522,10 @@
       <c r="A27" s="33"/>
       <c r="B27" s="14"/>
       <c r="C27" s="14"/>
-      <c r="D27" s="67"/>
-      <c r="E27" s="67"/>
+      <c r="D27" s="59"/>
+      <c r="E27" s="59"/>
       <c r="F27" s="33"/>
-      <c r="G27" s="70"/>
+      <c r="G27" s="62"/>
       <c r="H27" s="33" t="s">
         <v>37</v>
       </c>
@@ -3329,10 +3537,10 @@
       <c r="A28" s="33"/>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
-      <c r="D28" s="67"/>
-      <c r="E28" s="67"/>
+      <c r="D28" s="59"/>
+      <c r="E28" s="59"/>
       <c r="F28" s="33"/>
-      <c r="G28" s="70"/>
+      <c r="G28" s="62"/>
       <c r="I28" s="39" t="s">
         <v>62</v>
       </c>
@@ -3341,10 +3549,10 @@
       <c r="A29" s="33"/>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
-      <c r="D29" s="67"/>
-      <c r="E29" s="67"/>
+      <c r="D29" s="59"/>
+      <c r="E29" s="59"/>
       <c r="F29" s="33"/>
-      <c r="G29" s="70"/>
+      <c r="G29" s="62"/>
       <c r="I29" s="40" t="s">
         <v>81</v>
       </c>
@@ -3353,10 +3561,10 @@
       <c r="A30" s="33"/>
       <c r="B30" s="14"/>
       <c r="C30" s="14"/>
-      <c r="D30" s="67"/>
-      <c r="E30" s="67"/>
+      <c r="D30" s="59"/>
+      <c r="E30" s="59"/>
       <c r="F30" s="33"/>
-      <c r="G30" s="70"/>
+      <c r="G30" s="62"/>
       <c r="I30" s="43" t="s">
         <v>63</v>
       </c>
@@ -3386,14 +3594,14 @@
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="14"/>
-      <c r="D32" s="67" t="s">
+      <c r="D32" s="59" t="s">
         <v>113</v>
       </c>
-      <c r="E32" s="67"/>
+      <c r="E32" s="59"/>
       <c r="F32" s="33">
         <v>8</v>
       </c>
-      <c r="G32" s="70">
+      <c r="G32" s="62">
         <v>46275</v>
       </c>
       <c r="H32" s="33" t="s">
@@ -3407,10 +3615,10 @@
       <c r="A33" s="33"/>
       <c r="B33" s="14"/>
       <c r="C33" s="14"/>
-      <c r="D33" s="67"/>
-      <c r="E33" s="67"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
       <c r="F33" s="33"/>
-      <c r="G33" s="70"/>
+      <c r="G33" s="62"/>
       <c r="I33" s="41" t="s">
         <v>66</v>
       </c>
@@ -3419,10 +3627,10 @@
       <c r="A34" s="33"/>
       <c r="B34" s="14"/>
       <c r="C34" s="14"/>
-      <c r="D34" s="67"/>
-      <c r="E34" s="67"/>
+      <c r="D34" s="59"/>
+      <c r="E34" s="59"/>
       <c r="F34" s="33"/>
-      <c r="G34" s="70"/>
+      <c r="G34" s="62"/>
       <c r="H34" s="33" t="s">
         <v>115</v>
       </c>
@@ -3434,10 +3642,10 @@
       <c r="A35" s="33"/>
       <c r="B35" s="14"/>
       <c r="C35" s="14"/>
-      <c r="D35" s="67"/>
-      <c r="E35" s="67"/>
+      <c r="D35" s="59"/>
+      <c r="E35" s="59"/>
       <c r="F35" s="33"/>
-      <c r="G35" s="70"/>
+      <c r="G35" s="62"/>
       <c r="I35" s="41" t="s">
         <v>73</v>
       </c>
@@ -3446,10 +3654,10 @@
       <c r="A36" s="33"/>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
-      <c r="D36" s="67"/>
-      <c r="E36" s="67"/>
+      <c r="D36" s="59"/>
+      <c r="E36" s="59"/>
       <c r="F36" s="33"/>
-      <c r="G36" s="70"/>
+      <c r="G36" s="62"/>
       <c r="H36" s="33" t="s">
         <v>29</v>
       </c>
@@ -3461,10 +3669,10 @@
       <c r="A37" s="33"/>
       <c r="B37" s="14"/>
       <c r="C37" s="14"/>
-      <c r="D37" s="67"/>
-      <c r="E37" s="67"/>
+      <c r="D37" s="59"/>
+      <c r="E37" s="59"/>
       <c r="F37" s="33"/>
-      <c r="G37" s="70"/>
+      <c r="G37" s="62"/>
       <c r="I37" s="41" t="s">
         <v>75</v>
       </c>
@@ -3473,10 +3681,10 @@
       <c r="A38" s="33"/>
       <c r="B38" s="14"/>
       <c r="C38" s="14"/>
-      <c r="D38" s="67"/>
-      <c r="E38" s="67"/>
+      <c r="D38" s="59"/>
+      <c r="E38" s="59"/>
       <c r="F38" s="33"/>
-      <c r="G38" s="70"/>
+      <c r="G38" s="62"/>
       <c r="I38" s="41" t="s">
         <v>76</v>
       </c>
@@ -3485,10 +3693,10 @@
       <c r="A39" s="33"/>
       <c r="B39" s="14"/>
       <c r="C39" s="14"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="67"/>
+      <c r="D39" s="59"/>
+      <c r="E39" s="59"/>
       <c r="F39" s="33"/>
-      <c r="G39" s="70"/>
+      <c r="G39" s="62"/>
       <c r="I39" s="41" t="s">
         <v>77</v>
       </c>
@@ -3497,10 +3705,10 @@
       <c r="A40" s="33"/>
       <c r="B40" s="14"/>
       <c r="C40" s="14"/>
-      <c r="D40" s="67"/>
-      <c r="E40" s="67"/>
+      <c r="D40" s="59"/>
+      <c r="E40" s="59"/>
       <c r="F40" s="33"/>
-      <c r="G40" s="70"/>
+      <c r="G40" s="62"/>
       <c r="H40" s="33" t="s">
         <v>121</v>
       </c>
@@ -3512,10 +3720,10 @@
       <c r="A41" s="33"/>
       <c r="B41" s="14"/>
       <c r="C41" s="14"/>
-      <c r="D41" s="67"/>
-      <c r="E41" s="67"/>
+      <c r="D41" s="59"/>
+      <c r="E41" s="59"/>
       <c r="F41" s="33"/>
-      <c r="G41" s="70"/>
+      <c r="G41" s="62"/>
       <c r="I41" s="42" t="s">
         <v>123</v>
       </c>
@@ -3550,15 +3758,15 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D13B384-1725-40B5-B0F7-A3A77A0F68B1}">
-  <dimension ref="A1:J39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D13B384-1725-40B5-B0F7-A3A77A0F68B1}">
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.21875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="35.77734375" customWidth="1"/>
-    <col min="5" max="5" width="34.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="51.109375" customWidth="1"/>
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.5546875" bestFit="1" customWidth="1"/>
@@ -3567,29 +3775,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="68"/>
-      <c r="B1" s="59" t="s">
+      <c r="A1" s="60"/>
+      <c r="B1" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
       <c r="G1" s="56" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H1" s="56" t="s">
-        <v>161</v>
-      </c>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
+        <v>159</v>
+      </c>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" s="53" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C2" s="53" t="s">
         <v>132</v>
@@ -3601,36 +3809,36 @@
         <v>142</v>
       </c>
       <c r="F2" s="53" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G2" s="53" t="s">
         <v>106</v>
       </c>
       <c r="H2" s="53" t="s">
+        <v>158</v>
+      </c>
+      <c r="I2" s="53" t="s">
+        <v>161</v>
+      </c>
+      <c r="J2" s="53" t="s">
         <v>160</v>
-      </c>
-      <c r="I2" s="53" t="s">
-        <v>163</v>
-      </c>
-      <c r="J2" s="53" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="115.2">
       <c r="A3" s="33">
         <v>1</v>
       </c>
-      <c r="B3" s="72" t="s">
+      <c r="B3" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="C3" s="66" t="s">
+      <c r="C3" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="D3" s="66" t="s">
+      <c r="D3" s="58" t="s">
         <v>137</v>
       </c>
-      <c r="E3" s="66" t="s">
-        <v>146</v>
+      <c r="E3" s="58" t="s">
+        <v>145</v>
       </c>
       <c r="G3">
         <v>5</v>
@@ -3651,50 +3859,67 @@
       <c r="A4" s="33">
         <v>2</v>
       </c>
-      <c r="B4" s="72" t="s">
+      <c r="B4" s="64" t="s">
         <v>134</v>
       </c>
-      <c r="C4" s="66" t="s">
+      <c r="C4" s="58" t="s">
         <v>139</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="E4" s="66" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="316.8">
-      <c r="A5" s="33">
+        <v>146</v>
+      </c>
+      <c r="E4" s="58" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="13" customFormat="1" ht="409.2" customHeight="1">
+      <c r="A5" s="59">
         <v>3</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="31" t="s">
         <v>134</v>
       </c>
-      <c r="C5" s="71" t="s">
+      <c r="C5" s="63" t="s">
         <v>143</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="28.8">
+        <v>165</v>
+      </c>
+      <c r="E5" s="58" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="86.4">
       <c r="A6" s="33">
         <v>4</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="C6" s="66" t="s">
-        <v>157</v>
-      </c>
-      <c r="D6" s="1"/>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="33"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="1"/>
+      <c r="C6" s="58" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E6" s="58" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="86.4">
+      <c r="A7" s="77">
+        <v>5</v>
+      </c>
+      <c r="B7" s="78" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="79" t="s">
+        <v>168</v>
+      </c>
+      <c r="D7" s="80" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" s="81"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="33"/>
@@ -3720,199 +3945,12 @@
       <c r="C11" s="14"/>
       <c r="D11" s="31"/>
     </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="34"/>
-      <c r="B12" s="34"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="35" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="100.8">
-      <c r="A13" s="33">
-        <v>2</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="67" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="33"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="67"/>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="33"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="67"/>
-    </row>
-    <row r="16" spans="1:10">
-      <c r="A16" s="33"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="67"/>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="33"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="67"/>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="33"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="67"/>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="33"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="67"/>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="33"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="67"/>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="47"/>
-      <c r="B21" s="47"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="48" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="86.4">
-      <c r="A22" s="33">
-        <v>3</v>
-      </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="67" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="33"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="67"/>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="33"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="67"/>
-    </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="33"/>
-      <c r="B25" s="14"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="67"/>
-    </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="33"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="67"/>
-    </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="33"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="67"/>
-    </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="34"/>
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="35" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="86.4">
-      <c r="A29" s="33">
-        <v>4</v>
-      </c>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="67" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="33"/>
-      <c r="B30" s="14"/>
-      <c r="C30" s="14"/>
-      <c r="D30" s="67"/>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="33"/>
-      <c r="B31" s="14"/>
-      <c r="C31" s="14"/>
-      <c r="D31" s="67"/>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="33"/>
-      <c r="B32" s="14"/>
-      <c r="C32" s="14"/>
-      <c r="D32" s="67"/>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="33"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="67"/>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="33"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="67"/>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="33"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="67"/>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="33"/>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="67"/>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="33"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="67"/>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="33"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="67"/>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="47"/>
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="48" t="s">
-        <v>117</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3922,63 +3960,63 @@
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="73" t="s">
-        <v>156</v>
-      </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
+      <c r="A1" s="76" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="65" t="s">
+        <v>147</v>
+      </c>
+      <c r="B2" s="65" t="s">
+        <v>148</v>
+      </c>
+      <c r="C2" s="65" t="s">
         <v>149</v>
       </c>
-      <c r="B2" s="74" t="s">
+      <c r="D2" s="65" t="s">
         <v>150</v>
       </c>
-      <c r="C2" s="74" t="s">
+      <c r="E2" s="65" t="s">
         <v>151</v>
       </c>
-      <c r="D2" s="74" t="s">
+      <c r="F2" s="65" t="s">
         <v>152</v>
       </c>
-      <c r="E2" s="74" t="s">
+      <c r="G2" s="65" t="s">
         <v>153</v>
       </c>
-      <c r="F2" s="74" t="s">
-        <v>154</v>
-      </c>
-      <c r="G2" s="74" t="s">
-        <v>155</v>
-      </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="74">
+      <c r="A3" s="65">
         <v>1</v>
       </c>
-      <c r="B3" s="74">
+      <c r="B3" s="65">
         <v>2</v>
       </c>
-      <c r="C3" s="74">
+      <c r="C3" s="65">
         <f>A3+B3</f>
         <v>3</v>
       </c>
-      <c r="D3" s="74">
+      <c r="D3" s="65">
         <f t="shared" ref="D3:G3" si="0">B3+C3</f>
         <v>5</v>
       </c>
-      <c r="E3" s="74">
+      <c r="E3" s="65">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="F3" s="75">
+      <c r="F3" s="66">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="G3" s="76">
+      <c r="G3" s="67">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>

</xml_diff>